<commit_message>
docs(workbook): add Screen Actions rows for all legacy redirects
Adds one 'auto-redirect on page load' row per legacy alias / redirect
(30 rows). These are URLs that render nothing — they just redirect to
their canonical destination, so they only need a single Auto action row.

https://claude.ai/code/session_016suAGngRMLLHQX4wk1hDYn
</commit_message>
<xml_diff>
--- a/docs/workbook/emergent-energy-system-map.xlsx
+++ b/docs/workbook/emergent-energy-system-map.xlsx
@@ -5722,7 +5722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7706,6 +7706,1266 @@
       <c r="H47" s="2" t="inlineStr">
         <is>
           <t>work_items, work_item_assignments, tr_items, project_eng_approvals, project_eng_stages, eng_stage_templates, qc_item_instance, qc_template_item, qc_checklist, approvals, deliverables, ms_objects, project_info, users.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Execution Dashboard (legacy)</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>/dashboard</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /dashboard is immediately redirected to /gates. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /gates.</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Revenue (legacy)</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>/revenue</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /revenue is immediately redirected to /revenue-tracker. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /revenue-tracker.</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>COS Control (legacy)</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>/cos-control</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /cos-control is immediately redirected to /cos. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /cos.</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Cashflow Forecast (legacy)</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>/cashflow-forecast</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /cashflow-forecast is immediately redirected to /cashflow. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /cashflow.</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>My Tool (legacy)</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>/my-tool</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /my-tool is immediately redirected to /. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /.</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>My Tool / Week (legacy)</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>/my-tool/week</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /my-tool/week is immediately redirected to /my-work/calendar. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /my-work/calendar.</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>My Tool / Backlog (legacy)</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>/my-tool/backlog</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /my-tool/backlog is immediately redirected to /my-work/tasks. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /my-work/tasks.</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>My Tool / Settings (legacy)</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>/my-tool/settings</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /my-tool/settings is immediately redirected to /my-work/settings. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /my-work/settings.</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>My Tool / Help (legacy)</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>/my-tool/help</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /my-tool/help is immediately redirected to /. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /.</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>My Tool / Meetings (legacy)</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>/my-tool/meetings</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /my-tool/meetings is immediately redirected to /my-work/meetings. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /my-work/meetings.</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Company Priorities (legacy)</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>/company-priorities</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /company-priorities is immediately redirected to /priorities. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /priorities.</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Admin (legacy)</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>/admin</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /admin is immediately redirected to /admin/control-center. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /admin/control-center.</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Admin Legacy Utilities</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>/admin/legacy-utilities</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /admin/legacy-utilities is immediately redirected to /admin/control-center. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /admin/control-center.</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Exceptions (legacy)</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>/exceptions</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /exceptions is immediately redirected to /gates/exceptions. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /gates/exceptions.</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Project Lifecycle (legacy)</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>/project-lifecycle</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /project-lifecycle is immediately redirected to /lifecycle-board. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /lifecycle-board.</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Command Center (legacy)</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>/command-center</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /command-center is immediately redirected to /my-work. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /my-work.</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>SSEG (legacy)</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>/sseg</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /sseg is immediately redirected to /handover?tab=sseg. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /handover?tab=sseg.</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Quality Dashboard (project, legacy)</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>/quality/dashboard</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /quality/dashboard is immediately redirected to /quality. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /quality.</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>NCR List (legacy)</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>/quality/ncrs</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /quality/ncrs is immediately redirected to /quality. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /quality.</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>NCR Detail (legacy)</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>/quality/ncr/:id</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /quality/ncr/:id is immediately redirected to /quality. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /quality.</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Standups (alias)</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>/standups</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /standups is immediately redirected to /engineering/standup. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /engineering/standup.</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Teams Chats (alias)</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>/teams/chats</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /teams/chats is immediately redirected to /my-work/teams. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /my-work/teams.</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Collaboration Hub (alias)</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>/collaboration</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /collaboration is immediately redirected to /my-work. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /my-work.</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Collaboration Email (alias)</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>/collaboration/email</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /collaboration/email is immediately redirected to /my-work/email. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /my-work/email.</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Collaboration Teams (alias)</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>/collaboration/teams</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /collaboration/teams is immediately redirected to /my-work/teams. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /my-work/teams.</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>My Work Approvals (alias)</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>/my-work/approvals</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /my-work/approvals is immediately redirected to /my-work/tasks?source=approvals. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /my-work/tasks?source=approvals.</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>PM Deliverables (retired)</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>/pm/deliverables</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /pm/deliverables is immediately redirected to /pm/approvals. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /pm/approvals.</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Department Scores (alias)</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>/department-scores</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /department-scores is immediately redirected to /leaderboard?tab=departments. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /leaderboard?tab=departments.</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Procurement (alias)</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>/procurement</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /procurement is immediately redirected to /execution-board. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /execution-board.</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>HSE Compliance (alias)</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>/hse/compliance</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>(automatic on page load)</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>Legacy / alias URL. Any visit to /hse/compliance is immediately redirected to /hse?tab=compliance. Nothing is shown to the user and nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to /hse?tab=compliance.</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(workbook): full actions detail for projects.tsx (35 rows)
https://claude.ai/code/session_016suAGngRMLLHQX4wk1hDYn
</commit_message>
<xml_diff>
--- a/docs/workbook/emergent-energy-system-map.xlsx
+++ b/docs/workbook/emergent-energy-system-map.xlsx
@@ -5722,7 +5722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -8966,6 +8966,1476 @@
       <c r="H77" s="2" t="inlineStr">
         <is>
           <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/projects-summary</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>On load, fetches the master directory of every project with all columns needed for the table (name, phase, kWp, PM, PD, % complete, financial headline, dates, RAG, priority, escalation state).</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>Reads every project's live summary row.</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>Populates the main projects table.</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>project_info, project_execution_state, project_plan, dashboard_project_metrics, derived_project_kpis, priority_projects.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pm-assignable-users</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>On load, fetches the list of users who can be assigned as a PM, used to populate the PM dropdown in each row.</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>Reads users table filtered by PM-assignable role.</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>Populates the PM dropdown on each project row.</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>users, role_permissions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/priorities</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>On load, fetches the active company priorities for the priority-filter dropdown.</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Reads active priorities.</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>Populates the priority filter dropdown.</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>mytool_company_priorities, priority_projects, priority_derived_metrics (view).</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>(when priority filter selected) GET /api/priorities/:id</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>When you pick a specific priority from the filter, fetches that priority's detail so we can show only the projects linked to it.</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>Reads one priority's details.</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>Filters the projects table to just this priority's linked projects.</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>mytool_company_priorities, priority_projects.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>(when priority filter selected) GET /api/priorities/:id/detail</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>Sibling call to the priority-filter fetch — pulls enriched detail (linked projects and metrics).</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>Reads priority projects and metrics.</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>Feeds the priority-filter side panel.</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>priority_projects, derived_project_kpis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>(per project row) GET /api/projects-summary/:projectName/latest-update</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>When you hover / open a project row, fetches the latest PM weekly update for that project so we can show the tooltip / expanded row.</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>Reads the most recent weekly review for that project.</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>Populates the row's latest-update tooltip.</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>weekly_reviews.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>(per project row) GET /api/project-plan/:projectName</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>When you expand a project row, fetches its project plan (tasks) so PMs can see task-level completion.</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>Reads the project plan / work items for that project.</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>Populates the expanded-row task list.</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>work_items, project_plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>'Create Project' button</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>Navigates to the Project Create wizard to start a brand-new project.</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>Nothing on click.</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>Goes to /project-create.</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>None on click.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>'Export' button</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>Exports the current (filtered) project list as a CSV / Excel file for sharing outside the app.</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>Reads the already-loaded projects summary.</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>Triggers a browser download.</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>None (pure export of already-loaded data).</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>'Active projects' tab (`tab-active-projects`)</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>Tab</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>Switches the table to show only active (non-archived) projects.</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>Filters client-side, no new fetch.</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders table.</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>'Archived projects' tab (`tab-archived-projects`)</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>Tab</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>Switches the table to show only archived projects.</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>Filters client-side.</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders table.</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Phase filter (`select-phase-filter`)</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>Filter</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>Filters the table by project phase (Design, Construction, Commissioning, etc.).</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>Filters client-side.</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders table.</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>PM filter (`select-pm-filter`)</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>Filter</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>Filters the table by assigned PM.</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>Filters client-side.</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders table.</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>RAG filter (`select-rag-filter`)</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>Filter</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>Filters by RAG status: Red / Amber / Green.</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>Filters client-side.</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders table.</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Search box (`input-search`)</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>Filter</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>Free-text search across project names / codes / clients.</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>Filters client-side.</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders table.</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>Task search (`input-search-tasks`)</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>Filter</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>When a project row is expanded, free-text search inside that project's task list.</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>Filters the expanded task list client-side.</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders expanded row.</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Saved view picker (`select-view`)</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>Filter</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>Loads a saved column/filter/sort view.</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>Switches the local view config.</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders table.</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>'Clear' button</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>Resets all active filters to their defaults.</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>Clears local filter state.</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders table.</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Edit project name (`input-edit-project-name`)</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>Inline-edit of the project's display name.</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>Queues an update to the project row.</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>Commits on PATCH /api/project-info/:id.</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>project_info (update).</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Edit size kWp (`input-edit-size-kwp`)</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>Inline-edit of the project's size in kWp.</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>Queues an update.</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>Commits on PATCH /api/project-info/:id.</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>project_info (update).</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Edit phase (`select-edit-phase`)</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>Inline change of the project's current phase.</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>Queues a phase change.</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>Commits on PATCH /api/project-info/:id.</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>project_info (update), project_phase_history (insert).</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>Edit PM assignment (`select-edit-pm`)</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>Inline re-assignment of the PM owning the project.</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>Queues a PM change.</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>Commits on PATCH /api/project-info/:projectInfoId/assign-pm.</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>project_info (update), project_team_members (insert/update), audit_events (insert).</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Edit PD (`input-edit-pd`)</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>Inline re-assignment of the PD owning the project.</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>Queues a PD change.</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>Commits on PATCH /api/project-info/:id.</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>project_info (update).</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>Edit Construction Start date (`input-edit-construction-start`)</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>Inline edit of the construction start date.</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>Queues a date change.</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>Commits on PATCH /api/project-info/:id.</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>project_info (update).</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Edit Commissioning date (`input-edit-commissioning`)</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>Inline edit of the commissioning date.</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>Queues a date change.</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>Commits on PATCH /api/project-info/:id.</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>project_info (update).</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>Edit Client Handover date (`input-edit-client-handover`)</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>Inline edit of the client handover date.</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>Queues a date change.</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>Commits on PATCH /api/project-info/:id.</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>project_info (update).</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>Edit O&amp;M Handover date (`input-edit-om-handover`)</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>Inline edit of the operations &amp; maintenance handover date.</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>Queues a date change.</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>Commits on PATCH /api/project-info/:id.</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>project_info (update).</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>File upload (`input-file-upload`)</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>Upload a financial close document (PDF / Excel) and attach it to the project.</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>Sends the file to the financial-close upload endpoint.</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>Triggers GET /api/financial-close/upload handling.</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>project_financial_reviews (insert), sp_files (insert).</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>SharePoint link input (`input-sharepoint-link`)</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>Paste a SharePoint link instead of uploading a file.</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>Saves the link against the project.</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>Commits on PATCH /api/project-info/:id.</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>project_links (insert), project_info (update).</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>Not-applicable reason (`input-na-reason`)</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>If financial close isn't applicable for a project, record the reason.</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>Saves the reason against the project.</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>Commits on PATCH /api/project-info/:id.</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>project_info (update).</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>Saved view name (`input-view-name`)</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>Name for a new saved view when creating one.</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>Saves the view locally / to user prefs.</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>Updates local view list.</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>dashboard_preferences (update).</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>Inline % complete edit (in expanded task row)</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>Edits a task's % complete directly from the projects table.</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>Submits an override to the project plan.</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>POST /api/project-plan/overrides.</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>work_items (update), project_plan (update).</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>Escalate project (row action)</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>Flags or un-flags a project as escalated.</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>Posts an escalation change.</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>PATCH /api/projects-summary/:id/escalation.</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>project_info (update), audit_events (insert).</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>Project name link (each row)</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>Opens the detail page for that project.</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>Nothing on click.</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>Goes to /project/:projectName.</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>None on click.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>Projects (list)</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>/projects</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>PM chat icon (each row)</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>Opens the Teams chat group linked to that project.</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>Nothing on click.</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>Navigates to /my-work/teams (pre-filtered).</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>None on click.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(workbook): Batch 2 actions for 10 Engineering screens (37 rows)
https://claude.ai/code/session_016suAGngRMLLHQX4wk1hDYn
</commit_message>
<xml_diff>
--- a/docs/workbook/emergent-energy-system-map.xlsx
+++ b/docs/workbook/emergent-energy-system-map.xlsx
@@ -5722,7 +5722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H253"/>
+  <dimension ref="A1:H290"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -16356,6 +16356,1560 @@
         </is>
       </c>
       <c r="H253" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Dashboard</t>
+        </is>
+      </c>
+      <c r="B254" s="2" t="inlineStr">
+        <is>
+          <t>/engineering</t>
+        </is>
+      </c>
+      <c r="C254" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/mytool/company-priorities</t>
+        </is>
+      </c>
+      <c r="D254" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E254" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Engineering Dashboard screen calls /api/mytool/company-priorities to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F254" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G254" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Engineering Dashboard page.</t>
+        </is>
+      </c>
+      <c r="H254" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B255" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C255" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/eng/deliverables/{del.id}/acknowledge</t>
+        </is>
+      </c>
+      <c r="D255" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E255" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Engineering Tasks screen calls /api/eng/deliverables/{del.id}/acknowledge to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F255" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G255" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Engineering Tasks page.</t>
+        </is>
+      </c>
+      <c r="H255" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B256" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C256" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/eng/tasks/{task.id}/send-deliverable</t>
+        </is>
+      </c>
+      <c r="D256" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E256" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Engineering Tasks screen calls /api/eng/tasks/{task.id}/send-deliverable to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F256" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G256" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Engineering Tasks page.</t>
+        </is>
+      </c>
+      <c r="H256" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B257" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C257" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/eng/tasks/{task.id}/send-for-approval</t>
+        </is>
+      </c>
+      <c r="D257" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E257" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Engineering Tasks screen calls /api/eng/tasks/{task.id}/send-for-approval to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F257" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G257" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Engineering Tasks page.</t>
+        </is>
+      </c>
+      <c r="H257" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B258" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C258" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/projects-summary</t>
+        </is>
+      </c>
+      <c r="D258" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E258" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Engineering Tasks screen calls /api/projects-summary to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F258" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G258" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Engineering Tasks page.</t>
+        </is>
+      </c>
+      <c r="H258" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B259" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C259" s="2" t="inlineStr">
+        <is>
+          <t>`button-create-task` button</t>
+        </is>
+      </c>
+      <c r="D259" s="2" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+      <c r="E259" s="2" t="inlineStr">
+        <is>
+          <t>'Create task' button — triggers the 'create task' action on the Engineering Tasks screen.</t>
+        </is>
+      </c>
+      <c r="F259" s="2" t="inlineStr">
+        <is>
+          <t>Depends on the action; typically triggers a mutation or navigation (see Data Sources).</t>
+        </is>
+      </c>
+      <c r="G259" s="2" t="inlineStr">
+        <is>
+          <t>Varies — some close dialogs, some save, some navigate. See the page source for the exact onClick.</t>
+        </is>
+      </c>
+      <c r="H259" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B260" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C260" s="2" t="inlineStr">
+        <is>
+          <t>`button-submit-task` button</t>
+        </is>
+      </c>
+      <c r="D260" s="2" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+      <c r="E260" s="2" t="inlineStr">
+        <is>
+          <t>'Submit task' button — triggers the 'submit task' action on the Engineering Tasks screen.</t>
+        </is>
+      </c>
+      <c r="F260" s="2" t="inlineStr">
+        <is>
+          <t>Depends on the action; typically triggers a mutation or navigation (see Data Sources).</t>
+        </is>
+      </c>
+      <c r="G260" s="2" t="inlineStr">
+        <is>
+          <t>Varies — some close dialogs, some save, some navigate. See the page source for the exact onClick.</t>
+        </is>
+      </c>
+      <c r="H260" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B261" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C261" s="2" t="inlineStr">
+        <is>
+          <t>`input-comment` input</t>
+        </is>
+      </c>
+      <c r="D261" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E261" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'comment'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F261" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G261" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H261" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B262" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C262" s="2" t="inlineStr">
+        <is>
+          <t>`input-drawer-due-date` input</t>
+        </is>
+      </c>
+      <c r="D262" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E262" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'drawer due date'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F262" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G262" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H262" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B263" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C263" s="2" t="inlineStr">
+        <is>
+          <t>`input-drawer-start-date` input</t>
+        </is>
+      </c>
+      <c r="D263" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E263" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'drawer start date'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F263" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G263" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H263" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B264" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C264" s="2" t="inlineStr">
+        <is>
+          <t>`input-post-update` input</t>
+        </is>
+      </c>
+      <c r="D264" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E264" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'post update'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F264" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G264" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H264" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B265" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C265" s="2" t="inlineStr">
+        <is>
+          <t>`input-post-update-hold-reason` input</t>
+        </is>
+      </c>
+      <c r="D265" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E265" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'post update hold reason'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F265" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G265" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H265" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B266" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C266" s="2" t="inlineStr">
+        <is>
+          <t>`input-task-description` input</t>
+        </is>
+      </c>
+      <c r="D266" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E266" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'task description'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F266" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G266" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H266" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B267" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C267" s="2" t="inlineStr">
+        <is>
+          <t>`input-task-due` input</t>
+        </is>
+      </c>
+      <c r="D267" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E267" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'task due'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F267" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G267" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H267" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B268" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C268" s="2" t="inlineStr">
+        <is>
+          <t>`input-task-project` input</t>
+        </is>
+      </c>
+      <c r="D268" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E268" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'task project'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F268" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G268" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H268" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B269" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C269" s="2" t="inlineStr">
+        <is>
+          <t>`input-task-search` input</t>
+        </is>
+      </c>
+      <c r="D269" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E269" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'task search'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F269" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G269" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H269" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B270" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C270" s="2" t="inlineStr">
+        <is>
+          <t>`input-task-title` input</t>
+        </is>
+      </c>
+      <c r="D270" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E270" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'task title'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F270" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G270" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H270" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B271" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C271" s="2" t="inlineStr">
+        <is>
+          <t>`select-deliverable-recipient` selector</t>
+        </is>
+      </c>
+      <c r="D271" s="2" t="inlineStr">
+        <is>
+          <t>Form field / Filter</t>
+        </is>
+      </c>
+      <c r="E271" s="2" t="inlineStr">
+        <is>
+          <t>Dropdown for 'deliverable recipient'. Either filters the list client-side or captures a choice to submit.</t>
+        </is>
+      </c>
+      <c r="F271" s="2" t="inlineStr">
+        <is>
+          <t>Client-side filter, or submitted as part of a form.</t>
+        </is>
+      </c>
+      <c r="G271" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders or N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H271" s="2" t="inlineStr">
+        <is>
+          <t>See parent action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B272" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C272" s="2" t="inlineStr">
+        <is>
+          <t>`select-drawer-priority` selector</t>
+        </is>
+      </c>
+      <c r="D272" s="2" t="inlineStr">
+        <is>
+          <t>Form field / Filter</t>
+        </is>
+      </c>
+      <c r="E272" s="2" t="inlineStr">
+        <is>
+          <t>Dropdown for 'drawer priority'. Either filters the list client-side or captures a choice to submit.</t>
+        </is>
+      </c>
+      <c r="F272" s="2" t="inlineStr">
+        <is>
+          <t>Client-side filter, or submitted as part of a form.</t>
+        </is>
+      </c>
+      <c r="G272" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders or N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H272" s="2" t="inlineStr">
+        <is>
+          <t>See parent action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B273" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C273" s="2" t="inlineStr">
+        <is>
+          <t>`select-drawer-project` selector</t>
+        </is>
+      </c>
+      <c r="D273" s="2" t="inlineStr">
+        <is>
+          <t>Form field / Filter</t>
+        </is>
+      </c>
+      <c r="E273" s="2" t="inlineStr">
+        <is>
+          <t>Dropdown for 'drawer project'. Either filters the list client-side or captures a choice to submit.</t>
+        </is>
+      </c>
+      <c r="F273" s="2" t="inlineStr">
+        <is>
+          <t>Client-side filter, or submitted as part of a form.</t>
+        </is>
+      </c>
+      <c r="G273" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders or N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H273" s="2" t="inlineStr">
+        <is>
+          <t>See parent action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B274" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C274" s="2" t="inlineStr">
+        <is>
+          <t>`select-drawer-status` selector</t>
+        </is>
+      </c>
+      <c r="D274" s="2" t="inlineStr">
+        <is>
+          <t>Form field / Filter</t>
+        </is>
+      </c>
+      <c r="E274" s="2" t="inlineStr">
+        <is>
+          <t>Dropdown for 'drawer status'. Either filters the list client-side or captures a choice to submit.</t>
+        </is>
+      </c>
+      <c r="F274" s="2" t="inlineStr">
+        <is>
+          <t>Client-side filter, or submitted as part of a form.</t>
+        </is>
+      </c>
+      <c r="G274" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders or N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H274" s="2" t="inlineStr">
+        <is>
+          <t>See parent action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B275" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C275" s="2" t="inlineStr">
+        <is>
+          <t>`select-post-update-blocked-type` selector</t>
+        </is>
+      </c>
+      <c r="D275" s="2" t="inlineStr">
+        <is>
+          <t>Form field / Filter</t>
+        </is>
+      </c>
+      <c r="E275" s="2" t="inlineStr">
+        <is>
+          <t>Dropdown for 'post update blocked type'. Either filters the list client-side or captures a choice to submit.</t>
+        </is>
+      </c>
+      <c r="F275" s="2" t="inlineStr">
+        <is>
+          <t>Client-side filter, or submitted as part of a form.</t>
+        </is>
+      </c>
+      <c r="G275" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders or N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H275" s="2" t="inlineStr">
+        <is>
+          <t>See parent action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B276" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C276" s="2" t="inlineStr">
+        <is>
+          <t>`select-post-update-status` selector</t>
+        </is>
+      </c>
+      <c r="D276" s="2" t="inlineStr">
+        <is>
+          <t>Form field / Filter</t>
+        </is>
+      </c>
+      <c r="E276" s="2" t="inlineStr">
+        <is>
+          <t>Dropdown for 'post update status'. Either filters the list client-side or captures a choice to submit.</t>
+        </is>
+      </c>
+      <c r="F276" s="2" t="inlineStr">
+        <is>
+          <t>Client-side filter, or submitted as part of a form.</t>
+        </is>
+      </c>
+      <c r="G276" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders or N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H276" s="2" t="inlineStr">
+        <is>
+          <t>See parent action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B277" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C277" s="2" t="inlineStr">
+        <is>
+          <t>`select-task-assignee` selector</t>
+        </is>
+      </c>
+      <c r="D277" s="2" t="inlineStr">
+        <is>
+          <t>Form field / Filter</t>
+        </is>
+      </c>
+      <c r="E277" s="2" t="inlineStr">
+        <is>
+          <t>Dropdown for 'task assignee'. Either filters the list client-side or captures a choice to submit.</t>
+        </is>
+      </c>
+      <c r="F277" s="2" t="inlineStr">
+        <is>
+          <t>Client-side filter, or submitted as part of a form.</t>
+        </is>
+      </c>
+      <c r="G277" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders or N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H277" s="2" t="inlineStr">
+        <is>
+          <t>See parent action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Tasks</t>
+        </is>
+      </c>
+      <c r="B278" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/tasks</t>
+        </is>
+      </c>
+      <c r="C278" s="2" t="inlineStr">
+        <is>
+          <t>`select-task-priority` selector</t>
+        </is>
+      </c>
+      <c r="D278" s="2" t="inlineStr">
+        <is>
+          <t>Form field / Filter</t>
+        </is>
+      </c>
+      <c r="E278" s="2" t="inlineStr">
+        <is>
+          <t>Dropdown for 'task priority'. Either filters the list client-side or captures a choice to submit.</t>
+        </is>
+      </c>
+      <c r="F278" s="2" t="inlineStr">
+        <is>
+          <t>Client-side filter, or submitted as part of a form.</t>
+        </is>
+      </c>
+      <c r="G278" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders or N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H278" s="2" t="inlineStr">
+        <is>
+          <t>See parent action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Standup</t>
+        </is>
+      </c>
+      <c r="B279" s="2" t="inlineStr">
+        <is>
+          <t>/engineering/standup</t>
+        </is>
+      </c>
+      <c r="C279" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/standups/schedules</t>
+        </is>
+      </c>
+      <c r="D279" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E279" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Engineering Standup screen calls /api/standups/schedules to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F279" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G279" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Engineering Standup page.</t>
+        </is>
+      </c>
+      <c r="H279" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Monthly Report</t>
+        </is>
+      </c>
+      <c r="B280" s="2" t="inlineStr">
+        <is>
+          <t>/reports/engineering/monthly</t>
+        </is>
+      </c>
+      <c r="C280" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/engineering/monthly</t>
+        </is>
+      </c>
+      <c r="D280" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E280" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Engineering Monthly Report screen calls /api/reports/engineering/monthly to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F280" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G280" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Engineering Monthly Report page.</t>
+        </is>
+      </c>
+      <c r="H280" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Monthly Report</t>
+        </is>
+      </c>
+      <c r="B281" s="2" t="inlineStr">
+        <is>
+          <t>/reports/engineering/monthly</t>
+        </is>
+      </c>
+      <c r="C281" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/engineering/monthly?month={month}</t>
+        </is>
+      </c>
+      <c r="D281" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E281" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Engineering Monthly Report screen calls /api/reports/engineering/monthly?month={month} to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F281" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G281" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Engineering Monthly Report page.</t>
+        </is>
+      </c>
+      <c r="H281" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Monthly Report</t>
+        </is>
+      </c>
+      <c r="B282" s="2" t="inlineStr">
+        <is>
+          <t>/reports/engineering/monthly</t>
+        </is>
+      </c>
+      <c r="C282" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/engineering/monthly?month={prevMonth}</t>
+        </is>
+      </c>
+      <c r="D282" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E282" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Engineering Monthly Report screen calls /api/reports/engineering/monthly?month={prevMonth} to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F282" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G282" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Engineering Monthly Report page.</t>
+        </is>
+      </c>
+      <c r="H282" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Monthly History</t>
+        </is>
+      </c>
+      <c r="B283" s="2" t="inlineStr">
+        <is>
+          <t>/reports/engineering/monthly/history</t>
+        </is>
+      </c>
+      <c r="C283" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/engineering/monthly/history</t>
+        </is>
+      </c>
+      <c r="D283" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E283" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Engineering Monthly History screen calls /api/reports/engineering/monthly/history to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F283" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G283" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Engineering Monthly History page.</t>
+        </is>
+      </c>
+      <c r="H283" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Monthly Compare</t>
+        </is>
+      </c>
+      <c r="B284" s="2" t="inlineStr">
+        <is>
+          <t>/reports/engineering/monthly/compare</t>
+        </is>
+      </c>
+      <c r="C284" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/engineering/monthly/compare</t>
+        </is>
+      </c>
+      <c r="D284" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E284" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Engineering Monthly Compare screen calls /api/reports/engineering/monthly/compare to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F284" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G284" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Engineering Monthly Compare page.</t>
+        </is>
+      </c>
+      <c r="H284" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Monthly Compare</t>
+        </is>
+      </c>
+      <c r="B285" s="2" t="inlineStr">
+        <is>
+          <t>/reports/engineering/monthly/compare</t>
+        </is>
+      </c>
+      <c r="C285" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/engineering/monthly/compare?monthA={monthA}&amp;monthB={monthB}</t>
+        </is>
+      </c>
+      <c r="D285" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E285" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Engineering Monthly Compare screen calls /api/reports/engineering/monthly/compare?monthA={monthA}&amp;monthB={monthB} to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F285" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G285" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Engineering Monthly Compare page.</t>
+        </is>
+      </c>
+      <c r="H285" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Monthly Project</t>
+        </is>
+      </c>
+      <c r="B286" s="2" t="inlineStr">
+        <is>
+          <t>/reports/engineering/monthly/:month/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C286" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/engineering/monthly</t>
+        </is>
+      </c>
+      <c r="D286" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E286" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Engineering Monthly Project screen calls /api/reports/engineering/monthly to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F286" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G286" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Engineering Monthly Project page.</t>
+        </is>
+      </c>
+      <c r="H286" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Monthly Project</t>
+        </is>
+      </c>
+      <c r="B287" s="2" t="inlineStr">
+        <is>
+          <t>/reports/engineering/monthly/:month/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C287" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/engineering/monthly/{reportId}/drilldown?{q.toString()}</t>
+        </is>
+      </c>
+      <c r="D287" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E287" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Engineering Monthly Project screen calls /api/reports/engineering/monthly/{reportId}/drilldown?{q.toString()} to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F287" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G287" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Engineering Monthly Project page.</t>
+        </is>
+      </c>
+      <c r="H287" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Monthly Project</t>
+        </is>
+      </c>
+      <c r="B288" s="2" t="inlineStr">
+        <is>
+          <t>/reports/engineering/monthly/:month/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C288" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/engineering/monthly/{reportId}/project/{projectId}</t>
+        </is>
+      </c>
+      <c r="D288" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E288" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Engineering Monthly Project screen calls /api/reports/engineering/monthly/{reportId}/project/{projectId} to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F288" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G288" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Engineering Monthly Project page.</t>
+        </is>
+      </c>
+      <c r="H288" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Monthly Project</t>
+        </is>
+      </c>
+      <c r="B289" s="2" t="inlineStr">
+        <is>
+          <t>/reports/engineering/monthly/:month/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C289" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/engineering/monthly/project</t>
+        </is>
+      </c>
+      <c r="D289" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E289" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Engineering Monthly Project screen calls /api/reports/engineering/monthly/project to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F289" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G289" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Engineering Monthly Project page.</t>
+        </is>
+      </c>
+      <c r="H289" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Monthly Project</t>
+        </is>
+      </c>
+      <c r="B290" s="2" t="inlineStr">
+        <is>
+          <t>/reports/engineering/monthly/:month/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C290" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/engineering/monthly?month={month}</t>
+        </is>
+      </c>
+      <c r="D290" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E290" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Engineering Monthly Project screen calls /api/reports/engineering/monthly?month={month} to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F290" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G290" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Engineering Monthly Project page.</t>
+        </is>
+      </c>
+      <c r="H290" s="2" t="inlineStr">
         <is>
           <t>See Data Sources sheet for the handler + tables.</t>
         </is>

</xml_diff>

<commit_message>
docs(workbook): Batch 3 actions for 16 PM/PD/Handover screens (109 rows)
https://claude.ai/code/session_016suAGngRMLLHQX4wk1hDYn
</commit_message>
<xml_diff>
--- a/docs/workbook/emergent-energy-system-map.xlsx
+++ b/docs/workbook/emergent-energy-system-map.xlsx
@@ -5722,7 +5722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H290"/>
+  <dimension ref="A1:H399"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -17910,6 +17910,4584 @@
         </is>
       </c>
       <c r="H290" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="2" t="inlineStr">
+        <is>
+          <t>PM Dashboard</t>
+        </is>
+      </c>
+      <c r="B291" s="2" t="inlineStr">
+        <is>
+          <t>/pm-dashboard</t>
+        </is>
+      </c>
+      <c r="C291" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd-pm-handover/completed</t>
+        </is>
+      </c>
+      <c r="D291" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E291" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PM Dashboard screen calls /api/pd-pm-handover/completed to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F291" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G291" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PM Dashboard page.</t>
+        </is>
+      </c>
+      <c r="H291" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="2" t="inlineStr">
+        <is>
+          <t>PM Dashboard</t>
+        </is>
+      </c>
+      <c r="B292" s="2" t="inlineStr">
+        <is>
+          <t>/pm-dashboard</t>
+        </is>
+      </c>
+      <c r="C292" s="2" t="inlineStr">
+        <is>
+          <t>`tab-calendar` tab</t>
+        </is>
+      </c>
+      <c r="D292" s="2" t="inlineStr">
+        <is>
+          <t>Tab</t>
+        </is>
+      </c>
+      <c r="E292" s="2" t="inlineStr">
+        <is>
+          <t>Switches the PM Dashboard view to the 'calendar' tab.</t>
+        </is>
+      </c>
+      <c r="F292" s="2" t="inlineStr">
+        <is>
+          <t>Switches local state; may trigger a new query.</t>
+        </is>
+      </c>
+      <c r="G292" s="2" t="inlineStr">
+        <is>
+          <t>Stays on the same URL.</t>
+        </is>
+      </c>
+      <c r="H292" s="2" t="inlineStr">
+        <is>
+          <t>Depends on the tab's content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="2" t="inlineStr">
+        <is>
+          <t>PM Dashboard</t>
+        </is>
+      </c>
+      <c r="B293" s="2" t="inlineStr">
+        <is>
+          <t>/pm-dashboard</t>
+        </is>
+      </c>
+      <c r="C293" s="2" t="inlineStr">
+        <is>
+          <t>`tab-more-options` tab</t>
+        </is>
+      </c>
+      <c r="D293" s="2" t="inlineStr">
+        <is>
+          <t>Tab</t>
+        </is>
+      </c>
+      <c r="E293" s="2" t="inlineStr">
+        <is>
+          <t>Switches the PM Dashboard view to the 'more options' tab.</t>
+        </is>
+      </c>
+      <c r="F293" s="2" t="inlineStr">
+        <is>
+          <t>Switches local state; may trigger a new query.</t>
+        </is>
+      </c>
+      <c r="G293" s="2" t="inlineStr">
+        <is>
+          <t>Stays on the same URL.</t>
+        </is>
+      </c>
+      <c r="H293" s="2" t="inlineStr">
+        <is>
+          <t>Depends on the tab's content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="2" t="inlineStr">
+        <is>
+          <t>PM Dashboard</t>
+        </is>
+      </c>
+      <c r="B294" s="2" t="inlineStr">
+        <is>
+          <t>/pm-dashboard</t>
+        </is>
+      </c>
+      <c r="C294" s="2" t="inlineStr">
+        <is>
+          <t>`tab-overview` tab</t>
+        </is>
+      </c>
+      <c r="D294" s="2" t="inlineStr">
+        <is>
+          <t>Tab</t>
+        </is>
+      </c>
+      <c r="E294" s="2" t="inlineStr">
+        <is>
+          <t>Switches the PM Dashboard view to the 'overview' tab.</t>
+        </is>
+      </c>
+      <c r="F294" s="2" t="inlineStr">
+        <is>
+          <t>Switches local state; may trigger a new query.</t>
+        </is>
+      </c>
+      <c r="G294" s="2" t="inlineStr">
+        <is>
+          <t>Stays on the same URL.</t>
+        </is>
+      </c>
+      <c r="H294" s="2" t="inlineStr">
+        <is>
+          <t>Depends on the tab's content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="2" t="inlineStr">
+        <is>
+          <t>PM Dashboard</t>
+        </is>
+      </c>
+      <c r="B295" s="2" t="inlineStr">
+        <is>
+          <t>/pm-dashboard</t>
+        </is>
+      </c>
+      <c r="C295" s="2" t="inlineStr">
+        <is>
+          <t>`tab-priority` tab</t>
+        </is>
+      </c>
+      <c r="D295" s="2" t="inlineStr">
+        <is>
+          <t>Tab</t>
+        </is>
+      </c>
+      <c r="E295" s="2" t="inlineStr">
+        <is>
+          <t>Switches the PM Dashboard view to the 'priority' tab.</t>
+        </is>
+      </c>
+      <c r="F295" s="2" t="inlineStr">
+        <is>
+          <t>Switches local state; may trigger a new query.</t>
+        </is>
+      </c>
+      <c r="G295" s="2" t="inlineStr">
+        <is>
+          <t>Stays on the same URL.</t>
+        </is>
+      </c>
+      <c r="H295" s="2" t="inlineStr">
+        <is>
+          <t>Depends on the tab's content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Home</t>
+        </is>
+      </c>
+      <c r="B296" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go</t>
+        </is>
+      </c>
+      <c r="C296" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pm-otg/projects</t>
+        </is>
+      </c>
+      <c r="D296" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E296" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PM On-The-Go Home screen calls /api/pm-otg/projects to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F296" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G296" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PM On-The-Go Home page.</t>
+        </is>
+      </c>
+      <c r="H296" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B297" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C297" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/commissioning/{itemId}</t>
+        </is>
+      </c>
+      <c r="D297" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E297" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PM On-The-Go Project screen calls /api/commissioning/{itemId} to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F297" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G297" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PM On-The-Go Project page.</t>
+        </is>
+      </c>
+      <c r="H297" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B298" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C298" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pm-otg/projects/{projectId}/{endpoint}</t>
+        </is>
+      </c>
+      <c r="D298" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E298" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PM On-The-Go Project screen calls /api/pm-otg/projects/{projectId}/{endpoint} to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F298" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G298" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PM On-The-Go Project page.</t>
+        </is>
+      </c>
+      <c r="H298" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B299" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C299" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/procurement</t>
+        </is>
+      </c>
+      <c r="D299" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E299" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PM On-The-Go Project screen calls /api/procurement to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F299" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G299" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PM On-The-Go Project page.</t>
+        </is>
+      </c>
+      <c r="H299" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B300" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C300" s="2" t="inlineStr">
+        <is>
+          <t>`input-delay-days` input</t>
+        </is>
+      </c>
+      <c r="D300" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E300" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'delay days'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F300" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G300" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H300" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B301" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C301" s="2" t="inlineStr">
+        <is>
+          <t>`input-delay-description` input</t>
+        </is>
+      </c>
+      <c r="D301" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E301" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'delay description'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F301" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G301" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H301" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B302" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C302" s="2" t="inlineStr">
+        <is>
+          <t>`input-esc-description` input</t>
+        </is>
+      </c>
+      <c r="D302" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E302" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'esc description'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F302" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G302" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H302" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B303" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C303" s="2" t="inlineStr">
+        <is>
+          <t>`input-inv-amount` input</t>
+        </is>
+      </c>
+      <c r="D303" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E303" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'inv amount'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F303" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G303" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H303" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B304" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C304" s="2" t="inlineStr">
+        <is>
+          <t>`input-inv-number` input</t>
+        </is>
+      </c>
+      <c r="D304" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E304" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'inv number'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F304" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G304" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H304" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B305" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C305" s="2" t="inlineStr">
+        <is>
+          <t>`input-inv-po` input</t>
+        </is>
+      </c>
+      <c r="D305" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E305" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'inv po'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F305" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G305" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H305" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B306" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C306" s="2" t="inlineStr">
+        <is>
+          <t>`input-photo-caption` input</t>
+        </is>
+      </c>
+      <c r="D306" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E306" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'photo caption'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F306" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G306" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H306" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B307" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C307" s="2" t="inlineStr">
+        <is>
+          <t>`input-photo-event` input</t>
+        </is>
+      </c>
+      <c r="D307" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E307" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'photo event'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F307" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G307" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H307" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B308" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C308" s="2" t="inlineStr">
+        <is>
+          <t>`input-photo-file` input</t>
+        </is>
+      </c>
+      <c r="D308" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E308" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'photo file'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F308" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G308" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H308" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B309" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C309" s="2" t="inlineStr">
+        <is>
+          <t>`input-po-amount` input</t>
+        </is>
+      </c>
+      <c r="D309" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E309" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'po amount'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F309" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G309" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H309" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B310" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C310" s="2" t="inlineStr">
+        <is>
+          <t>`input-po-description` input</t>
+        </is>
+      </c>
+      <c r="D310" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E310" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'po description'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F310" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G310" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H310" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B311" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C311" s="2" t="inlineStr">
+        <is>
+          <t>`input-po-number` input</t>
+        </is>
+      </c>
+      <c r="D311" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E311" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'po number'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F311" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G311" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H311" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B312" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C312" s="2" t="inlineStr">
+        <is>
+          <t>`input-po-supplier` input</t>
+        </is>
+      </c>
+      <c r="D312" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E312" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'po supplier'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F312" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G312" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H312" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B313" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C313" s="2" t="inlineStr">
+        <is>
+          <t>`input-proc-cost` input</t>
+        </is>
+      </c>
+      <c r="D313" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E313" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'proc cost'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F313" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G313" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H313" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B314" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C314" s="2" t="inlineStr">
+        <is>
+          <t>`input-proc-date` input</t>
+        </is>
+      </c>
+      <c r="D314" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E314" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'proc date'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F314" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G314" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H314" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B315" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C315" s="2" t="inlineStr">
+        <is>
+          <t>`input-proc-description` input</t>
+        </is>
+      </c>
+      <c r="D315" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E315" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'proc description'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F315" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G315" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H315" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B316" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C316" s="2" t="inlineStr">
+        <is>
+          <t>`input-proc-title` input</t>
+        </is>
+      </c>
+      <c r="D316" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E316" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'proc title'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F316" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G316" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H316" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B317" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C317" s="2" t="inlineStr">
+        <is>
+          <t>`input-progress-notes` input</t>
+        </is>
+      </c>
+      <c r="D317" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E317" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'progress notes'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F317" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G317" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H317" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B318" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C318" s="2" t="inlineStr">
+        <is>
+          <t>`input-risk-description` input</t>
+        </is>
+      </c>
+      <c r="D318" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E318" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'risk description'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F318" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G318" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H318" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B319" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C319" s="2" t="inlineStr">
+        <is>
+          <t>`input-risk-mitigation` input</t>
+        </is>
+      </c>
+      <c r="D319" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E319" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'risk mitigation'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F319" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G319" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H319" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B320" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C320" s="2" t="inlineStr">
+        <is>
+          <t>`input-sv-date` input</t>
+        </is>
+      </c>
+      <c r="D320" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E320" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'sv date'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F320" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G320" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H320" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B321" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C321" s="2" t="inlineStr">
+        <is>
+          <t>`input-sv-notes` input</t>
+        </is>
+      </c>
+      <c r="D321" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E321" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'sv notes'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F321" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G321" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H321" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B322" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C322" s="2" t="inlineStr">
+        <is>
+          <t>`input-sv-photos` input</t>
+        </is>
+      </c>
+      <c r="D322" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E322" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'sv photos'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F322" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G322" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H322" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B323" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C323" s="2" t="inlineStr">
+        <is>
+          <t>`input-vo-amount` input</t>
+        </is>
+      </c>
+      <c r="D323" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E323" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'vo amount'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F323" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G323" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H323" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B324" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C324" s="2" t="inlineStr">
+        <is>
+          <t>`input-vo-description` input</t>
+        </is>
+      </c>
+      <c r="D324" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E324" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'vo description'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F324" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G324" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H324" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B325" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C325" s="2" t="inlineStr">
+        <is>
+          <t>`input-vo-justification` input</t>
+        </is>
+      </c>
+      <c r="D325" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E325" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'vo justification'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F325" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G325" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H325" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B326" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C326" s="2" t="inlineStr">
+        <is>
+          <t>`select-delay-impact` selector</t>
+        </is>
+      </c>
+      <c r="D326" s="2" t="inlineStr">
+        <is>
+          <t>Form field / Filter</t>
+        </is>
+      </c>
+      <c r="E326" s="2" t="inlineStr">
+        <is>
+          <t>Dropdown for 'delay impact'. Either filters the list client-side or captures a choice to submit.</t>
+        </is>
+      </c>
+      <c r="F326" s="2" t="inlineStr">
+        <is>
+          <t>Client-side filter, or submitted as part of a form.</t>
+        </is>
+      </c>
+      <c r="G326" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders or N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H326" s="2" t="inlineStr">
+        <is>
+          <t>See parent action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B327" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C327" s="2" t="inlineStr">
+        <is>
+          <t>`select-esc-level` selector</t>
+        </is>
+      </c>
+      <c r="D327" s="2" t="inlineStr">
+        <is>
+          <t>Form field / Filter</t>
+        </is>
+      </c>
+      <c r="E327" s="2" t="inlineStr">
+        <is>
+          <t>Dropdown for 'esc level'. Either filters the list client-side or captures a choice to submit.</t>
+        </is>
+      </c>
+      <c r="F327" s="2" t="inlineStr">
+        <is>
+          <t>Client-side filter, or submitted as part of a form.</t>
+        </is>
+      </c>
+      <c r="G327" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders or N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H327" s="2" t="inlineStr">
+        <is>
+          <t>See parent action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B328" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C328" s="2" t="inlineStr">
+        <is>
+          <t>`select-esc-urgency` selector</t>
+        </is>
+      </c>
+      <c r="D328" s="2" t="inlineStr">
+        <is>
+          <t>Form field / Filter</t>
+        </is>
+      </c>
+      <c r="E328" s="2" t="inlineStr">
+        <is>
+          <t>Dropdown for 'esc urgency'. Either filters the list client-side or captures a choice to submit.</t>
+        </is>
+      </c>
+      <c r="F328" s="2" t="inlineStr">
+        <is>
+          <t>Client-side filter, or submitted as part of a form.</t>
+        </is>
+      </c>
+      <c r="G328" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders or N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H328" s="2" t="inlineStr">
+        <is>
+          <t>See parent action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B329" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C329" s="2" t="inlineStr">
+        <is>
+          <t>`select-proc-category` selector</t>
+        </is>
+      </c>
+      <c r="D329" s="2" t="inlineStr">
+        <is>
+          <t>Form field / Filter</t>
+        </is>
+      </c>
+      <c r="E329" s="2" t="inlineStr">
+        <is>
+          <t>Dropdown for 'proc category'. Either filters the list client-side or captures a choice to submit.</t>
+        </is>
+      </c>
+      <c r="F329" s="2" t="inlineStr">
+        <is>
+          <t>Client-side filter, or submitted as part of a form.</t>
+        </is>
+      </c>
+      <c r="G329" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders or N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H329" s="2" t="inlineStr">
+        <is>
+          <t>See parent action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B330" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C330" s="2" t="inlineStr">
+        <is>
+          <t>`select-risk-severity` selector</t>
+        </is>
+      </c>
+      <c r="D330" s="2" t="inlineStr">
+        <is>
+          <t>Form field / Filter</t>
+        </is>
+      </c>
+      <c r="E330" s="2" t="inlineStr">
+        <is>
+          <t>Dropdown for 'risk severity'. Either filters the list client-side or captures a choice to submit.</t>
+        </is>
+      </c>
+      <c r="F330" s="2" t="inlineStr">
+        <is>
+          <t>Client-side filter, or submitted as part of a form.</t>
+        </is>
+      </c>
+      <c r="G330" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders or N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H330" s="2" t="inlineStr">
+        <is>
+          <t>See parent action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="2" t="inlineStr">
+        <is>
+          <t>PM On-The-Go Project</t>
+        </is>
+      </c>
+      <c r="B331" s="2" t="inlineStr">
+        <is>
+          <t>/pm/on-the-go/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C331" s="2" t="inlineStr">
+        <is>
+          <t>`select-sv-weather` selector</t>
+        </is>
+      </c>
+      <c r="D331" s="2" t="inlineStr">
+        <is>
+          <t>Form field / Filter</t>
+        </is>
+      </c>
+      <c r="E331" s="2" t="inlineStr">
+        <is>
+          <t>Dropdown for 'sv weather'. Either filters the list client-side or captures a choice to submit.</t>
+        </is>
+      </c>
+      <c r="F331" s="2" t="inlineStr">
+        <is>
+          <t>Client-side filter, or submitted as part of a form.</t>
+        </is>
+      </c>
+      <c r="G331" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders or N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H331" s="2" t="inlineStr">
+        <is>
+          <t>See parent action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="2" t="inlineStr">
+        <is>
+          <t>PM Handover Review</t>
+        </is>
+      </c>
+      <c r="B332" s="2" t="inlineStr">
+        <is>
+          <t>/pm/handover-review</t>
+        </is>
+      </c>
+      <c r="C332" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd-pm-handover/submitted</t>
+        </is>
+      </c>
+      <c r="D332" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E332" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PM Handover Review screen calls /api/pd-pm-handover/submitted to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F332" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G332" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PM Handover Review page.</t>
+        </is>
+      </c>
+      <c r="H332" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="2" t="inlineStr">
+        <is>
+          <t>PM Monthly Report</t>
+        </is>
+      </c>
+      <c r="B333" s="2" t="inlineStr">
+        <is>
+          <t>/reports/pm/monthly</t>
+        </is>
+      </c>
+      <c r="C333" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/pm/monthly</t>
+        </is>
+      </c>
+      <c r="D333" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E333" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PM Monthly Report screen calls /api/reports/pm/monthly to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F333" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G333" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PM Monthly Report page.</t>
+        </is>
+      </c>
+      <c r="H333" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="2" t="inlineStr">
+        <is>
+          <t>PM Monthly Report</t>
+        </is>
+      </c>
+      <c r="B334" s="2" t="inlineStr">
+        <is>
+          <t>/reports/pm/monthly</t>
+        </is>
+      </c>
+      <c r="C334" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/pm/monthly/compare</t>
+        </is>
+      </c>
+      <c r="D334" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E334" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PM Monthly Report screen calls /api/reports/pm/monthly/compare to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F334" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G334" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PM Monthly Report page.</t>
+        </is>
+      </c>
+      <c r="H334" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="2" t="inlineStr">
+        <is>
+          <t>PM Monthly Report</t>
+        </is>
+      </c>
+      <c r="B335" s="2" t="inlineStr">
+        <is>
+          <t>/reports/pm/monthly</t>
+        </is>
+      </c>
+      <c r="C335" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/pm/monthly/compare?monthA={previousMonth}&amp;monthB={month}</t>
+        </is>
+      </c>
+      <c r="D335" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E335" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PM Monthly Report screen calls /api/reports/pm/monthly/compare?monthA={previousMonth}&amp;monthB={month} to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F335" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G335" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PM Monthly Report page.</t>
+        </is>
+      </c>
+      <c r="H335" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="2" t="inlineStr">
+        <is>
+          <t>PM Monthly Report</t>
+        </is>
+      </c>
+      <c r="B336" s="2" t="inlineStr">
+        <is>
+          <t>/reports/pm/monthly</t>
+        </is>
+      </c>
+      <c r="C336" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/pm/monthly?month={month}</t>
+        </is>
+      </c>
+      <c r="D336" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E336" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PM Monthly Report screen calls /api/reports/pm/monthly?month={month} to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F336" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G336" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PM Monthly Report page.</t>
+        </is>
+      </c>
+      <c r="H336" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="2" t="inlineStr">
+        <is>
+          <t>PM Monthly Report History</t>
+        </is>
+      </c>
+      <c r="B337" s="2" t="inlineStr">
+        <is>
+          <t>/reports/pm/monthly/history</t>
+        </is>
+      </c>
+      <c r="C337" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/pm/monthly/history</t>
+        </is>
+      </c>
+      <c r="D337" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E337" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PM Monthly Report History screen calls /api/reports/pm/monthly/history to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F337" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G337" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PM Monthly Report History page.</t>
+        </is>
+      </c>
+      <c r="H337" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="2" t="inlineStr">
+        <is>
+          <t>PM Monthly Report Compare</t>
+        </is>
+      </c>
+      <c r="B338" s="2" t="inlineStr">
+        <is>
+          <t>/reports/pm/monthly/compare</t>
+        </is>
+      </c>
+      <c r="C338" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/pm/monthly/compare</t>
+        </is>
+      </c>
+      <c r="D338" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E338" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PM Monthly Report Compare screen calls /api/reports/pm/monthly/compare to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F338" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G338" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PM Monthly Report Compare page.</t>
+        </is>
+      </c>
+      <c r="H338" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="2" t="inlineStr">
+        <is>
+          <t>PM Monthly Report Compare</t>
+        </is>
+      </c>
+      <c r="B339" s="2" t="inlineStr">
+        <is>
+          <t>/reports/pm/monthly/compare</t>
+        </is>
+      </c>
+      <c r="C339" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/pm/monthly/compare?monthA={monthA}&amp;monthB={monthB}</t>
+        </is>
+      </c>
+      <c r="D339" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E339" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PM Monthly Report Compare screen calls /api/reports/pm/monthly/compare?monthA={monthA}&amp;monthB={monthB} to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F339" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G339" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PM Monthly Report Compare page.</t>
+        </is>
+      </c>
+      <c r="H339" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="2" t="inlineStr">
+        <is>
+          <t>PM Monthly Report Project</t>
+        </is>
+      </c>
+      <c r="B340" s="2" t="inlineStr">
+        <is>
+          <t>/reports/pm/monthly/:month/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C340" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/pm/monthly</t>
+        </is>
+      </c>
+      <c r="D340" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E340" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PM Monthly Report Project screen calls /api/reports/pm/monthly to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F340" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G340" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PM Monthly Report Project page.</t>
+        </is>
+      </c>
+      <c r="H340" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="2" t="inlineStr">
+        <is>
+          <t>PM Monthly Report Project</t>
+        </is>
+      </c>
+      <c r="B341" s="2" t="inlineStr">
+        <is>
+          <t>/reports/pm/monthly/:month/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C341" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/pm/monthly/{reportId}/drilldown?{q.toString()}</t>
+        </is>
+      </c>
+      <c r="D341" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E341" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PM Monthly Report Project screen calls /api/reports/pm/monthly/{reportId}/drilldown?{q.toString()} to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F341" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G341" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PM Monthly Report Project page.</t>
+        </is>
+      </c>
+      <c r="H341" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="2" t="inlineStr">
+        <is>
+          <t>PM Monthly Report Project</t>
+        </is>
+      </c>
+      <c r="B342" s="2" t="inlineStr">
+        <is>
+          <t>/reports/pm/monthly/:month/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C342" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/pm/monthly/{reportId}/project/{projectId}</t>
+        </is>
+      </c>
+      <c r="D342" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E342" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PM Monthly Report Project screen calls /api/reports/pm/monthly/{reportId}/project/{projectId} to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F342" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G342" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PM Monthly Report Project page.</t>
+        </is>
+      </c>
+      <c r="H342" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="2" t="inlineStr">
+        <is>
+          <t>PM Monthly Report Project</t>
+        </is>
+      </c>
+      <c r="B343" s="2" t="inlineStr">
+        <is>
+          <t>/reports/pm/monthly/:month/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C343" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/pm/monthly/project</t>
+        </is>
+      </c>
+      <c r="D343" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E343" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PM Monthly Report Project screen calls /api/reports/pm/monthly/project to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F343" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G343" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PM Monthly Report Project page.</t>
+        </is>
+      </c>
+      <c r="H343" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="2" t="inlineStr">
+        <is>
+          <t>PM Monthly Report Project</t>
+        </is>
+      </c>
+      <c r="B344" s="2" t="inlineStr">
+        <is>
+          <t>/reports/pm/monthly/:month/project/:projectId</t>
+        </is>
+      </c>
+      <c r="C344" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/reports/pm/monthly?month={month}</t>
+        </is>
+      </c>
+      <c r="D344" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E344" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PM Monthly Report Project screen calls /api/reports/pm/monthly?month={month} to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F344" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G344" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PM Monthly Report Project page.</t>
+        </is>
+      </c>
+      <c r="H344" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="2" t="inlineStr">
+        <is>
+          <t>PD Dashboard</t>
+        </is>
+      </c>
+      <c r="B345" s="2" t="inlineStr">
+        <is>
+          <t>/pd</t>
+        </is>
+      </c>
+      <c r="C345" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd-pm-handover/control</t>
+        </is>
+      </c>
+      <c r="D345" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E345" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD Dashboard screen calls /api/pd-pm-handover/control to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F345" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G345" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD Dashboard page.</t>
+        </is>
+      </c>
+      <c r="H345" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="2" t="inlineStr">
+        <is>
+          <t>PD Dashboard</t>
+        </is>
+      </c>
+      <c r="B346" s="2" t="inlineStr">
+        <is>
+          <t>/pd</t>
+        </is>
+      </c>
+      <c r="C346" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd/dashboard</t>
+        </is>
+      </c>
+      <c r="D346" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E346" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD Dashboard screen calls /api/pd/dashboard to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F346" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G346" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD Dashboard page.</t>
+        </is>
+      </c>
+      <c r="H346" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="2" t="inlineStr">
+        <is>
+          <t>PD Dashboard</t>
+        </is>
+      </c>
+      <c r="B347" s="2" t="inlineStr">
+        <is>
+          <t>/pd</t>
+        </is>
+      </c>
+      <c r="C347" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd/pipeline</t>
+        </is>
+      </c>
+      <c r="D347" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E347" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD Dashboard screen calls /api/pd/pipeline to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F347" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G347" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD Dashboard page.</t>
+        </is>
+      </c>
+      <c r="H347" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="2" t="inlineStr">
+        <is>
+          <t>PD Dashboard</t>
+        </is>
+      </c>
+      <c r="B348" s="2" t="inlineStr">
+        <is>
+          <t>/pd</t>
+        </is>
+      </c>
+      <c r="C348" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd/tickets</t>
+        </is>
+      </c>
+      <c r="D348" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E348" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD Dashboard screen calls /api/pd/tickets to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F348" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G348" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD Dashboard page.</t>
+        </is>
+      </c>
+      <c r="H348" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="2" t="inlineStr">
+        <is>
+          <t>PD Dashboard</t>
+        </is>
+      </c>
+      <c r="B349" s="2" t="inlineStr">
+        <is>
+          <t>/pd</t>
+        </is>
+      </c>
+      <c r="C349" s="2" t="inlineStr">
+        <is>
+          <t>`link-handover-control` link</t>
+        </is>
+      </c>
+      <c r="D349" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="E349" s="2" t="inlineStr">
+        <is>
+          <t>Navigates to the 'handover control' destination.</t>
+        </is>
+      </c>
+      <c r="F349" s="2" t="inlineStr">
+        <is>
+          <t>Nothing on click.</t>
+        </is>
+      </c>
+      <c r="G349" s="2" t="inlineStr">
+        <is>
+          <t>Varies — see source.</t>
+        </is>
+      </c>
+      <c r="H349" s="2" t="inlineStr">
+        <is>
+          <t>None on click.</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="2" t="inlineStr">
+        <is>
+          <t>PD Dashboard</t>
+        </is>
+      </c>
+      <c r="B350" s="2" t="inlineStr">
+        <is>
+          <t>/pd</t>
+        </is>
+      </c>
+      <c r="C350" s="2" t="inlineStr">
+        <is>
+          <t>`link-view-all-tickets` link</t>
+        </is>
+      </c>
+      <c r="D350" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="E350" s="2" t="inlineStr">
+        <is>
+          <t>Navigates to the 'view all tickets' destination.</t>
+        </is>
+      </c>
+      <c r="F350" s="2" t="inlineStr">
+        <is>
+          <t>Nothing on click.</t>
+        </is>
+      </c>
+      <c r="G350" s="2" t="inlineStr">
+        <is>
+          <t>Varies — see source.</t>
+        </is>
+      </c>
+      <c r="H350" s="2" t="inlineStr">
+        <is>
+          <t>None on click.</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="2" t="inlineStr">
+        <is>
+          <t>PD Tickets</t>
+        </is>
+      </c>
+      <c r="B351" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets</t>
+        </is>
+      </c>
+      <c r="C351" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd/tickets</t>
+        </is>
+      </c>
+      <c r="D351" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E351" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD Tickets screen calls /api/pd/tickets to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F351" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G351" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD Tickets page.</t>
+        </is>
+      </c>
+      <c r="H351" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B352" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C352" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd/clients</t>
+        </is>
+      </c>
+      <c r="D352" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E352" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD Ticket Create screen calls /api/pd/clients to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F352" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G352" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD Ticket Create page.</t>
+        </is>
+      </c>
+      <c r="H352" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B353" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C353" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd/dashboard</t>
+        </is>
+      </c>
+      <c r="D353" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E353" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD Ticket Create screen calls /api/pd/dashboard to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F353" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G353" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD Ticket Create page.</t>
+        </is>
+      </c>
+      <c r="H353" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B354" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C354" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd/projects/search</t>
+        </is>
+      </c>
+      <c r="D354" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E354" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD Ticket Create screen calls /api/pd/projects/search to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F354" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G354" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD Ticket Create page.</t>
+        </is>
+      </c>
+      <c r="H354" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B355" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C355" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd/tickets</t>
+        </is>
+      </c>
+      <c r="D355" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E355" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD Ticket Create screen calls /api/pd/tickets to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F355" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G355" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD Ticket Create page.</t>
+        </is>
+      </c>
+      <c r="H355" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B356" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C356" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd/users</t>
+        </is>
+      </c>
+      <c r="D356" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E356" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD Ticket Create screen calls /api/pd/users to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F356" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G356" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD Ticket Create page.</t>
+        </is>
+      </c>
+      <c r="H356" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B357" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C357" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/projects/similar-names</t>
+        </is>
+      </c>
+      <c r="D357" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E357" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD Ticket Create screen calls /api/projects/similar-names to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F357" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G357" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD Ticket Create page.</t>
+        </is>
+      </c>
+      <c r="H357" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B358" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C358" s="2" t="inlineStr">
+        <is>
+          <t>`input-battery-size` input</t>
+        </is>
+      </c>
+      <c r="D358" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E358" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'battery size'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F358" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G358" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H358" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B359" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C359" s="2" t="inlineStr">
+        <is>
+          <t>`input-client-search` input</t>
+        </is>
+      </c>
+      <c r="D359" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E359" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'client search'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F359" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G359" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H359" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B360" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C360" s="2" t="inlineStr">
+        <is>
+          <t>`input-comments` input</t>
+        </is>
+      </c>
+      <c r="D360" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E360" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'comments'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F360" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G360" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H360" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B361" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C361" s="2" t="inlineStr">
+        <is>
+          <t>`input-due-date` input</t>
+        </is>
+      </c>
+      <c r="D361" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E361" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'due date'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F361" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G361" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H361" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B362" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C362" s="2" t="inlineStr">
+        <is>
+          <t>`input-gps` input</t>
+        </is>
+      </c>
+      <c r="D362" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E362" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'gps'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F362" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G362" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H362" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B363" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C363" s="2" t="inlineStr">
+        <is>
+          <t>`input-inspection-link` input</t>
+        </is>
+      </c>
+      <c r="D363" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E363" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'inspection link'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F363" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G363" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H363" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B364" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C364" s="2" t="inlineStr">
+        <is>
+          <t>`input-new-client-name` input</t>
+        </is>
+      </c>
+      <c r="D364" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E364" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'new client name'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F364" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G364" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H364" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B365" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C365" s="2" t="inlineStr">
+        <is>
+          <t>`input-new-project-name` input</t>
+        </is>
+      </c>
+      <c r="D365" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E365" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'new project name'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F365" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G365" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H365" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B366" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C366" s="2" t="inlineStr">
+        <is>
+          <t>`input-project-search` input</t>
+        </is>
+      </c>
+      <c r="D366" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E366" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'project search'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F366" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G366" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H366" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B367" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C367" s="2" t="inlineStr">
+        <is>
+          <t>`input-site-name` input</t>
+        </is>
+      </c>
+      <c r="D367" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E367" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'site name'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F367" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G367" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H367" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B368" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C368" s="2" t="inlineStr">
+        <is>
+          <t>`input-size-kwp` input</t>
+        </is>
+      </c>
+      <c r="D368" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E368" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'size kwp'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F368" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G368" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H368" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B369" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C369" s="2" t="inlineStr">
+        <is>
+          <t>`input-working-schedule` input</t>
+        </is>
+      </c>
+      <c r="D369" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E369" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'working schedule'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F369" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G369" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H369" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B370" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C370" s="2" t="inlineStr">
+        <is>
+          <t>`select-designer` selector</t>
+        </is>
+      </c>
+      <c r="D370" s="2" t="inlineStr">
+        <is>
+          <t>Form field / Filter</t>
+        </is>
+      </c>
+      <c r="E370" s="2" t="inlineStr">
+        <is>
+          <t>Dropdown for 'designer'. Either filters the list client-side or captures a choice to submit.</t>
+        </is>
+      </c>
+      <c r="F370" s="2" t="inlineStr">
+        <is>
+          <t>Client-side filter, or submitted as part of a form.</t>
+        </is>
+      </c>
+      <c r="G370" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders or N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H370" s="2" t="inlineStr">
+        <is>
+          <t>See parent action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B371" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C371" s="2" t="inlineStr">
+        <is>
+          <t>`select-funding-type` selector</t>
+        </is>
+      </c>
+      <c r="D371" s="2" t="inlineStr">
+        <is>
+          <t>Form field / Filter</t>
+        </is>
+      </c>
+      <c r="E371" s="2" t="inlineStr">
+        <is>
+          <t>Dropdown for 'funding type'. Either filters the list client-side or captures a choice to submit.</t>
+        </is>
+      </c>
+      <c r="F371" s="2" t="inlineStr">
+        <is>
+          <t>Client-side filter, or submitted as part of a form.</t>
+        </is>
+      </c>
+      <c r="G371" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders or N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H371" s="2" t="inlineStr">
+        <is>
+          <t>See parent action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B372" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C372" s="2" t="inlineStr">
+        <is>
+          <t>`select-priority` selector</t>
+        </is>
+      </c>
+      <c r="D372" s="2" t="inlineStr">
+        <is>
+          <t>Form field / Filter</t>
+        </is>
+      </c>
+      <c r="E372" s="2" t="inlineStr">
+        <is>
+          <t>Dropdown for 'priority'. Either filters the list client-side or captures a choice to submit.</t>
+        </is>
+      </c>
+      <c r="F372" s="2" t="inlineStr">
+        <is>
+          <t>Client-side filter, or submitted as part of a form.</t>
+        </is>
+      </c>
+      <c r="G372" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders or N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H372" s="2" t="inlineStr">
+        <is>
+          <t>See parent action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B373" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C373" s="2" t="inlineStr">
+        <is>
+          <t>`select-province` selector</t>
+        </is>
+      </c>
+      <c r="D373" s="2" t="inlineStr">
+        <is>
+          <t>Form field / Filter</t>
+        </is>
+      </c>
+      <c r="E373" s="2" t="inlineStr">
+        <is>
+          <t>Dropdown for 'province'. Either filters the list client-side or captures a choice to submit.</t>
+        </is>
+      </c>
+      <c r="F373" s="2" t="inlineStr">
+        <is>
+          <t>Client-side filter, or submitted as part of a form.</t>
+        </is>
+      </c>
+      <c r="G373" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders or N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H373" s="2" t="inlineStr">
+        <is>
+          <t>See parent action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Create</t>
+        </is>
+      </c>
+      <c r="B374" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/create</t>
+        </is>
+      </c>
+      <c r="C374" s="2" t="inlineStr">
+        <is>
+          <t>`select-request-type` selector</t>
+        </is>
+      </c>
+      <c r="D374" s="2" t="inlineStr">
+        <is>
+          <t>Form field / Filter</t>
+        </is>
+      </c>
+      <c r="E374" s="2" t="inlineStr">
+        <is>
+          <t>Dropdown for 'request type'. Either filters the list client-side or captures a choice to submit.</t>
+        </is>
+      </c>
+      <c r="F374" s="2" t="inlineStr">
+        <is>
+          <t>Client-side filter, or submitted as part of a form.</t>
+        </is>
+      </c>
+      <c r="G374" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders or N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H374" s="2" t="inlineStr">
+        <is>
+          <t>See parent action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Detail</t>
+        </is>
+      </c>
+      <c r="B375" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/:id</t>
+        </is>
+      </c>
+      <c r="C375" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/eng/tasks</t>
+        </is>
+      </c>
+      <c r="D375" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E375" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD Ticket Detail screen calls /api/eng/tasks to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F375" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G375" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD Ticket Detail page.</t>
+        </is>
+      </c>
+      <c r="H375" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Detail</t>
+        </is>
+      </c>
+      <c r="B376" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/:id</t>
+        </is>
+      </c>
+      <c r="C376" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd/tickets</t>
+        </is>
+      </c>
+      <c r="D376" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E376" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD Ticket Detail screen calls /api/pd/tickets to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F376" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G376" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD Ticket Detail page.</t>
+        </is>
+      </c>
+      <c r="H376" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Detail</t>
+        </is>
+      </c>
+      <c r="B377" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/:id</t>
+        </is>
+      </c>
+      <c r="C377" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd/users</t>
+        </is>
+      </c>
+      <c r="D377" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E377" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD Ticket Detail screen calls /api/pd/users to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F377" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G377" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD Ticket Detail page.</t>
+        </is>
+      </c>
+      <c r="H377" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Detail</t>
+        </is>
+      </c>
+      <c r="B378" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/:id</t>
+        </is>
+      </c>
+      <c r="C378" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/projects</t>
+        </is>
+      </c>
+      <c r="D378" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E378" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD Ticket Detail screen calls /api/projects to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F378" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G378" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD Ticket Detail page.</t>
+        </is>
+      </c>
+      <c r="H378" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Detail</t>
+        </is>
+      </c>
+      <c r="B379" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/:id</t>
+        </is>
+      </c>
+      <c r="C379" s="2" t="inlineStr">
+        <is>
+          <t>`input-new-engineering-ticket-description` input</t>
+        </is>
+      </c>
+      <c r="D379" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E379" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'new engineering ticket description'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F379" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G379" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H379" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Detail</t>
+        </is>
+      </c>
+      <c r="B380" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/:id</t>
+        </is>
+      </c>
+      <c r="C380" s="2" t="inlineStr">
+        <is>
+          <t>`input-new-engineering-ticket-due-date` input</t>
+        </is>
+      </c>
+      <c r="D380" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E380" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'new engineering ticket due date'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F380" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G380" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H380" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Detail</t>
+        </is>
+      </c>
+      <c r="B381" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/:id</t>
+        </is>
+      </c>
+      <c r="C381" s="2" t="inlineStr">
+        <is>
+          <t>`input-new-engineering-ticket-title` input</t>
+        </is>
+      </c>
+      <c r="D381" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E381" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'new engineering ticket title'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F381" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G381" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H381" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="2" t="inlineStr">
+        <is>
+          <t>PD Ticket Detail</t>
+        </is>
+      </c>
+      <c r="B382" s="2" t="inlineStr">
+        <is>
+          <t>/pd/tickets/:id</t>
+        </is>
+      </c>
+      <c r="C382" s="2" t="inlineStr">
+        <is>
+          <t>`link-to-project` link</t>
+        </is>
+      </c>
+      <c r="D382" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="E382" s="2" t="inlineStr">
+        <is>
+          <t>Navigates to the 'to project' destination.</t>
+        </is>
+      </c>
+      <c r="F382" s="2" t="inlineStr">
+        <is>
+          <t>Nothing on click.</t>
+        </is>
+      </c>
+      <c r="G382" s="2" t="inlineStr">
+        <is>
+          <t>Varies — see source.</t>
+        </is>
+      </c>
+      <c r="H382" s="2" t="inlineStr">
+        <is>
+          <t>None on click.</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="2" t="inlineStr">
+        <is>
+          <t>PD Reports</t>
+        </is>
+      </c>
+      <c r="B383" s="2" t="inlineStr">
+        <is>
+          <t>/pd/reports</t>
+        </is>
+      </c>
+      <c r="C383" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd/reports</t>
+        </is>
+      </c>
+      <c r="D383" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E383" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD Reports screen calls /api/pd/reports to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F383" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G383" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD Reports page.</t>
+        </is>
+      </c>
+      <c r="H383" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="2" t="inlineStr">
+        <is>
+          <t>PD→PM Handover v2</t>
+        </is>
+      </c>
+      <c r="B384" s="2" t="inlineStr">
+        <is>
+          <t>/pd/handover/:projectId</t>
+        </is>
+      </c>
+      <c r="C384" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/lessons-learnt?projectType={encodeURIComponent(tabData.projectType)}&amp;limit=3</t>
+        </is>
+      </c>
+      <c r="D384" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E384" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD→PM Handover v2 screen calls /api/lessons-learnt?projectType={encodeURIComponent(tabData.projectType)}&amp;limit=3 to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F384" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G384" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD→PM Handover v2 page.</t>
+        </is>
+      </c>
+      <c r="H384" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="2" t="inlineStr">
+        <is>
+          <t>PD→PM Handover v2</t>
+        </is>
+      </c>
+      <c r="B385" s="2" t="inlineStr">
+        <is>
+          <t>/pd/handover/:projectId</t>
+        </is>
+      </c>
+      <c r="C385" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd-pm-handover/{projectId}</t>
+        </is>
+      </c>
+      <c r="D385" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E385" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD→PM Handover v2 screen calls /api/pd-pm-handover/{projectId} to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F385" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G385" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD→PM Handover v2 page.</t>
+        </is>
+      </c>
+      <c r="H385" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="2" t="inlineStr">
+        <is>
+          <t>PD→PM Handover v2</t>
+        </is>
+      </c>
+      <c r="B386" s="2" t="inlineStr">
+        <is>
+          <t>/pd/handover/:projectId</t>
+        </is>
+      </c>
+      <c r="C386" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd-pm-handover/{projectId}/accept</t>
+        </is>
+      </c>
+      <c r="D386" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E386" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD→PM Handover v2 screen calls /api/pd-pm-handover/{projectId}/accept to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F386" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G386" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD→PM Handover v2 page.</t>
+        </is>
+      </c>
+      <c r="H386" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="2" t="inlineStr">
+        <is>
+          <t>PD→PM Handover v2</t>
+        </is>
+      </c>
+      <c r="B387" s="2" t="inlineStr">
+        <is>
+          <t>/pd/handover/:projectId</t>
+        </is>
+      </c>
+      <c r="C387" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd-pm-handover/{projectId}/draft</t>
+        </is>
+      </c>
+      <c r="D387" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E387" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD→PM Handover v2 screen calls /api/pd-pm-handover/{projectId}/draft to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F387" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G387" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD→PM Handover v2 page.</t>
+        </is>
+      </c>
+      <c r="H387" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="2" t="inlineStr">
+        <is>
+          <t>PD→PM Handover v2</t>
+        </is>
+      </c>
+      <c r="B388" s="2" t="inlineStr">
+        <is>
+          <t>/pd/handover/:projectId</t>
+        </is>
+      </c>
+      <c r="C388" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd-pm-handover/{projectId}/pd-sign-off</t>
+        </is>
+      </c>
+      <c r="D388" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E388" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD→PM Handover v2 screen calls /api/pd-pm-handover/{projectId}/pd-sign-off to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F388" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G388" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD→PM Handover v2 page.</t>
+        </is>
+      </c>
+      <c r="H388" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="2" t="inlineStr">
+        <is>
+          <t>PD→PM Handover v2</t>
+        </is>
+      </c>
+      <c r="B389" s="2" t="inlineStr">
+        <is>
+          <t>/pd/handover/:projectId</t>
+        </is>
+      </c>
+      <c r="C389" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd-pm-handover/{projectId}/pm-sign-off</t>
+        </is>
+      </c>
+      <c r="D389" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E389" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD→PM Handover v2 screen calls /api/pd-pm-handover/{projectId}/pm-sign-off to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F389" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G389" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD→PM Handover v2 page.</t>
+        </is>
+      </c>
+      <c r="H389" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="2" t="inlineStr">
+        <is>
+          <t>PD→PM Handover v2</t>
+        </is>
+      </c>
+      <c r="B390" s="2" t="inlineStr">
+        <is>
+          <t>/pd/handover/:projectId</t>
+        </is>
+      </c>
+      <c r="C390" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd-pm-handover/{projectId}/reject</t>
+        </is>
+      </c>
+      <c r="D390" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E390" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD→PM Handover v2 screen calls /api/pd-pm-handover/{projectId}/reject to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F390" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G390" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD→PM Handover v2 page.</t>
+        </is>
+      </c>
+      <c r="H390" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="2" t="inlineStr">
+        <is>
+          <t>PD→PM Handover v2</t>
+        </is>
+      </c>
+      <c r="B391" s="2" t="inlineStr">
+        <is>
+          <t>/pd/handover/:projectId</t>
+        </is>
+      </c>
+      <c r="C391" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd-pm-handover/{projectId}/stakeholders</t>
+        </is>
+      </c>
+      <c r="D391" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E391" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD→PM Handover v2 screen calls /api/pd-pm-handover/{projectId}/stakeholders to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F391" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G391" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD→PM Handover v2 page.</t>
+        </is>
+      </c>
+      <c r="H391" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="2" t="inlineStr">
+        <is>
+          <t>PD→PM Handover v2</t>
+        </is>
+      </c>
+      <c r="B392" s="2" t="inlineStr">
+        <is>
+          <t>/pd/handover/:projectId</t>
+        </is>
+      </c>
+      <c r="C392" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd-pm-handover/{projectId}/stakeholders/{id}</t>
+        </is>
+      </c>
+      <c r="D392" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E392" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD→PM Handover v2 screen calls /api/pd-pm-handover/{projectId}/stakeholders/{id} to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F392" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G392" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD→PM Handover v2 page.</t>
+        </is>
+      </c>
+      <c r="H392" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="2" t="inlineStr">
+        <is>
+          <t>PD→PM Handover v2</t>
+        </is>
+      </c>
+      <c r="B393" s="2" t="inlineStr">
+        <is>
+          <t>/pd/handover/:projectId</t>
+        </is>
+      </c>
+      <c r="C393" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd-pm-handover/{projectId}/submit</t>
+        </is>
+      </c>
+      <c r="D393" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E393" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD→PM Handover v2 screen calls /api/pd-pm-handover/{projectId}/submit to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F393" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G393" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD→PM Handover v2 page.</t>
+        </is>
+      </c>
+      <c r="H393" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="2" t="inlineStr">
+        <is>
+          <t>PD→PM Handover v2</t>
+        </is>
+      </c>
+      <c r="B394" s="2" t="inlineStr">
+        <is>
+          <t>/pd/handover/:projectId</t>
+        </is>
+      </c>
+      <c r="C394" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd-pm-handover/control</t>
+        </is>
+      </c>
+      <c r="D394" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E394" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD→PM Handover v2 screen calls /api/pd-pm-handover/control to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F394" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G394" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD→PM Handover v2 page.</t>
+        </is>
+      </c>
+      <c r="H394" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="2" t="inlineStr">
+        <is>
+          <t>PD→PM Handover v2</t>
+        </is>
+      </c>
+      <c r="B395" s="2" t="inlineStr">
+        <is>
+          <t>/pd/handover/:projectId</t>
+        </is>
+      </c>
+      <c r="C395" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/projects-summary</t>
+        </is>
+      </c>
+      <c r="D395" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E395" s="2" t="inlineStr">
+        <is>
+          <t>On load, the PD→PM Handover v2 screen calls /api/projects-summary to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F395" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G395" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the PD→PM Handover v2 page.</t>
+        </is>
+      </c>
+      <c r="H395" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="2" t="inlineStr">
+        <is>
+          <t>Handover Control</t>
+        </is>
+      </c>
+      <c r="B396" s="2" t="inlineStr">
+        <is>
+          <t>/handover-control</t>
+        </is>
+      </c>
+      <c r="C396" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/pd-pm-handover/control</t>
+        </is>
+      </c>
+      <c r="D396" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E396" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Handover Control screen calls /api/pd-pm-handover/control to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F396" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G396" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Handover Control page.</t>
+        </is>
+      </c>
+      <c r="H396" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="2" t="inlineStr">
+        <is>
+          <t>Handover Dashboard</t>
+        </is>
+      </c>
+      <c r="B397" s="2" t="inlineStr">
+        <is>
+          <t>/handover</t>
+        </is>
+      </c>
+      <c r="C397" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/handover/packs</t>
+        </is>
+      </c>
+      <c r="D397" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E397" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Handover Dashboard screen calls /api/handover/packs to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F397" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G397" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Handover Dashboard page.</t>
+        </is>
+      </c>
+      <c r="H397" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="2" t="inlineStr">
+        <is>
+          <t>Handover Dashboard</t>
+        </is>
+      </c>
+      <c r="B398" s="2" t="inlineStr">
+        <is>
+          <t>/handover</t>
+        </is>
+      </c>
+      <c r="C398" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/handover/sseg</t>
+        </is>
+      </c>
+      <c r="D398" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E398" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Handover Dashboard screen calls /api/handover/sseg to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F398" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G398" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Handover Dashboard page.</t>
+        </is>
+      </c>
+      <c r="H398" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="2" t="inlineStr">
+        <is>
+          <t>Handover Dashboard</t>
+        </is>
+      </c>
+      <c r="B399" s="2" t="inlineStr">
+        <is>
+          <t>/handover</t>
+        </is>
+      </c>
+      <c r="C399" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/sseg-applications</t>
+        </is>
+      </c>
+      <c r="D399" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E399" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Handover Dashboard screen calls /api/sseg-applications to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F399" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G399" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Handover Dashboard page.</t>
+        </is>
+      </c>
+      <c r="H399" s="2" t="inlineStr">
         <is>
           <t>See Data Sources sheet for the handler + tables.</t>
         </is>

</xml_diff>

<commit_message>
docs(workbook): Batch 5 actions for Quality/HSE/Commissioning (12 rows)
https://claude.ai/code/session_016suAGngRMLLHQX4wk1hDYn
</commit_message>
<xml_diff>
--- a/docs/workbook/emergent-energy-system-map.xlsx
+++ b/docs/workbook/emergent-energy-system-map.xlsx
@@ -5722,7 +5722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H546"/>
+  <dimension ref="A1:H558"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -28662,6 +28662,510 @@
         </is>
       </c>
       <c r="H546" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" s="2" t="inlineStr">
+        <is>
+          <t>QM Dashboard (Quality)</t>
+        </is>
+      </c>
+      <c r="B547" s="2" t="inlineStr">
+        <is>
+          <t>/quality</t>
+        </is>
+      </c>
+      <c r="C547" s="2" t="inlineStr">
+        <is>
+          <t>`input-qm-project-search` input</t>
+        </is>
+      </c>
+      <c r="D547" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E547" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'qm project search'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F547" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G547" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H547" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" s="2" t="inlineStr">
+        <is>
+          <t>QM Dashboard (Quality)</t>
+        </is>
+      </c>
+      <c r="B548" s="2" t="inlineStr">
+        <is>
+          <t>/quality</t>
+        </is>
+      </c>
+      <c r="C548" s="2" t="inlineStr">
+        <is>
+          <t>`input-qm-search` input</t>
+        </is>
+      </c>
+      <c r="D548" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E548" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'qm search'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F548" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G548" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H548" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" s="2" t="inlineStr">
+        <is>
+          <t>QM Dashboard (Quality)</t>
+        </is>
+      </c>
+      <c r="B549" s="2" t="inlineStr">
+        <is>
+          <t>/quality</t>
+        </is>
+      </c>
+      <c r="C549" s="2" t="inlineStr">
+        <is>
+          <t>`input-warning-reason` input</t>
+        </is>
+      </c>
+      <c r="D549" s="2" t="inlineStr">
+        <is>
+          <t>Form field</t>
+        </is>
+      </c>
+      <c r="E549" s="2" t="inlineStr">
+        <is>
+          <t>Input for 'warning reason'. Captures the value to be submitted.</t>
+        </is>
+      </c>
+      <c r="F549" s="2" t="inlineStr">
+        <is>
+          <t>Submitted as part of a form mutation.</t>
+        </is>
+      </c>
+      <c r="G549" s="2" t="inlineStr">
+        <is>
+          <t>N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H549" s="2" t="inlineStr">
+        <is>
+          <t>Saved by the parent form's mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" s="2" t="inlineStr">
+        <is>
+          <t>QM Dashboard (Quality)</t>
+        </is>
+      </c>
+      <c r="B550" s="2" t="inlineStr">
+        <is>
+          <t>/quality</t>
+        </is>
+      </c>
+      <c r="C550" s="2" t="inlineStr">
+        <is>
+          <t>`select-qm-project` selector</t>
+        </is>
+      </c>
+      <c r="D550" s="2" t="inlineStr">
+        <is>
+          <t>Form field / Filter</t>
+        </is>
+      </c>
+      <c r="E550" s="2" t="inlineStr">
+        <is>
+          <t>Dropdown for 'qm project'. Either filters the list client-side or captures a choice to submit.</t>
+        </is>
+      </c>
+      <c r="F550" s="2" t="inlineStr">
+        <is>
+          <t>Client-side filter, or submitted as part of a form.</t>
+        </is>
+      </c>
+      <c r="G550" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders or N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H550" s="2" t="inlineStr">
+        <is>
+          <t>See parent action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" s="2" t="inlineStr">
+        <is>
+          <t>QM Dashboard (Quality)</t>
+        </is>
+      </c>
+      <c r="B551" s="2" t="inlineStr">
+        <is>
+          <t>/quality</t>
+        </is>
+      </c>
+      <c r="C551" s="2" t="inlineStr">
+        <is>
+          <t>`select-status-filter` selector</t>
+        </is>
+      </c>
+      <c r="D551" s="2" t="inlineStr">
+        <is>
+          <t>Form field / Filter</t>
+        </is>
+      </c>
+      <c r="E551" s="2" t="inlineStr">
+        <is>
+          <t>Dropdown for 'status filter'. Either filters the list client-side or captures a choice to submit.</t>
+        </is>
+      </c>
+      <c r="F551" s="2" t="inlineStr">
+        <is>
+          <t>Client-side filter, or submitted as part of a form.</t>
+        </is>
+      </c>
+      <c r="G551" s="2" t="inlineStr">
+        <is>
+          <t>Re-renders or N/A until submit.</t>
+        </is>
+      </c>
+      <c r="H551" s="2" t="inlineStr">
+        <is>
+          <t>See parent action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" s="2" t="inlineStr">
+        <is>
+          <t>HSE Dashboard</t>
+        </is>
+      </c>
+      <c r="B552" s="2" t="inlineStr">
+        <is>
+          <t>/hse</t>
+        </is>
+      </c>
+      <c r="C552" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/hse/corrective-actions</t>
+        </is>
+      </c>
+      <c r="D552" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E552" s="2" t="inlineStr">
+        <is>
+          <t>On load, the HSE Dashboard screen calls /api/hse/corrective-actions to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F552" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G552" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the HSE Dashboard page.</t>
+        </is>
+      </c>
+      <c r="H552" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" s="2" t="inlineStr">
+        <is>
+          <t>HSE Dashboard</t>
+        </is>
+      </c>
+      <c r="B553" s="2" t="inlineStr">
+        <is>
+          <t>/hse</t>
+        </is>
+      </c>
+      <c r="C553" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/hse/incidents</t>
+        </is>
+      </c>
+      <c r="D553" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E553" s="2" t="inlineStr">
+        <is>
+          <t>On load, the HSE Dashboard screen calls /api/hse/incidents to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F553" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G553" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the HSE Dashboard page.</t>
+        </is>
+      </c>
+      <c r="H553" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" s="2" t="inlineStr">
+        <is>
+          <t>HSE Dashboard</t>
+        </is>
+      </c>
+      <c r="B554" s="2" t="inlineStr">
+        <is>
+          <t>/hse</t>
+        </is>
+      </c>
+      <c r="C554" s="2" t="inlineStr">
+        <is>
+          <t>PATCH /api/hse/incidents/{id}</t>
+        </is>
+      </c>
+      <c r="D554" s="2" t="inlineStr">
+        <is>
+          <t>Mutation</t>
+        </is>
+      </c>
+      <c r="E554" s="2" t="inlineStr">
+        <is>
+          <t>Sends a PATCH to /api/hse/incidents/{id} when the user saves / triggers an action on this screen.</t>
+        </is>
+      </c>
+      <c r="F554" s="2" t="inlineStr">
+        <is>
+          <t>Writes to the server.</t>
+        </is>
+      </c>
+      <c r="G554" s="2" t="inlineStr">
+        <is>
+          <t>Usually re-queries the affected lists on success, shows a toast.</t>
+        </is>
+      </c>
+      <c r="H554" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" s="2" t="inlineStr">
+        <is>
+          <t>HSE Dashboard</t>
+        </is>
+      </c>
+      <c r="B555" s="2" t="inlineStr">
+        <is>
+          <t>/hse</t>
+        </is>
+      </c>
+      <c r="C555" s="2" t="inlineStr">
+        <is>
+          <t>POST /api/hse/incidents</t>
+        </is>
+      </c>
+      <c r="D555" s="2" t="inlineStr">
+        <is>
+          <t>Mutation</t>
+        </is>
+      </c>
+      <c r="E555" s="2" t="inlineStr">
+        <is>
+          <t>Sends a POST to /api/hse/incidents when the user saves / triggers an action on this screen.</t>
+        </is>
+      </c>
+      <c r="F555" s="2" t="inlineStr">
+        <is>
+          <t>Writes to the server.</t>
+        </is>
+      </c>
+      <c r="G555" s="2" t="inlineStr">
+        <is>
+          <t>Usually re-queries the affected lists on success, shows a toast.</t>
+        </is>
+      </c>
+      <c r="H555" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" s="2" t="inlineStr">
+        <is>
+          <t>Commissioning Dashboard</t>
+        </is>
+      </c>
+      <c r="B556" s="2" t="inlineStr">
+        <is>
+          <t>/commissioning-dashboard</t>
+        </is>
+      </c>
+      <c r="C556" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/commissioning-dashboard/{projectId}</t>
+        </is>
+      </c>
+      <c r="D556" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E556" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Commissioning Dashboard screen calls /api/commissioning-dashboard/{projectId} to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F556" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G556" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Commissioning Dashboard page.</t>
+        </is>
+      </c>
+      <c r="H556" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" s="2" t="inlineStr">
+        <is>
+          <t>Commissioning Dashboard</t>
+        </is>
+      </c>
+      <c r="B557" s="2" t="inlineStr">
+        <is>
+          <t>/commissioning-dashboard</t>
+        </is>
+      </c>
+      <c r="C557" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/commissioning-dashboard/{projectId}/refresh</t>
+        </is>
+      </c>
+      <c r="D557" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E557" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Commissioning Dashboard screen calls /api/commissioning-dashboard/{projectId}/refresh to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F557" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G557" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Commissioning Dashboard page.</t>
+        </is>
+      </c>
+      <c r="H557" s="2" t="inlineStr">
+        <is>
+          <t>See Data Sources sheet for the handler + tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" s="2" t="inlineStr">
+        <is>
+          <t>Commissioning Dashboard</t>
+        </is>
+      </c>
+      <c r="B558" s="2" t="inlineStr">
+        <is>
+          <t>/commissioning-dashboard</t>
+        </is>
+      </c>
+      <c r="C558" s="2" t="inlineStr">
+        <is>
+          <t>(page load) GET /api/commissioning-dashboard/{projectId}/upload</t>
+        </is>
+      </c>
+      <c r="D558" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E558" s="2" t="inlineStr">
+        <is>
+          <t>On load, the Commissioning Dashboard screen calls /api/commissioning-dashboard/{projectId}/upload to fetch data it needs to render.</t>
+        </is>
+      </c>
+      <c r="F558" s="2" t="inlineStr">
+        <is>
+          <t>Read from the server.</t>
+        </is>
+      </c>
+      <c r="G558" s="2" t="inlineStr">
+        <is>
+          <t>Populates a section of the Commissioning Dashboard page.</t>
+        </is>
+      </c>
+      <c r="H558" s="2" t="inlineStr">
         <is>
           <t>See Data Sources sheet for the handler + tables.</t>
         </is>

</xml_diff>